<commit_message>
Change the detector box
</commit_message>
<xml_diff>
--- a/Teacher_Detailed_Attendance.xlsx
+++ b/Teacher_Detailed_Attendance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -589,6 +589,216 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20:12:23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>20:13:49</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>20:14:05</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0:00:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>20:18:34</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>20:18:49</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0:00:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>20:19:08</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
enhance code with new library and excel
</commit_message>
<xml_diff>
--- a/Teacher_Detailed_Attendance.xlsx
+++ b/Teacher_Detailed_Attendance.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -50,7 +49,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,8 +412,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -456,12 +455,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06:27:20</t>
+          <t>03:53:03</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -489,12 +488,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06:27:47</t>
+          <t>03:53:36</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -514,20 +513,24 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0:00:33</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06:32:40</t>
+          <t>03:53:49</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,12 +558,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06:33:11</t>
+          <t>03:54:01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -585,19 +588,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0:00:30</t>
+          <t>0:00:11</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20:12:23</t>
+          <t>03:54:30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -620,318 +623,9 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>20:13:49</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-001</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Ubada Hussain</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>20:14:05</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-001</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Ubada Hussain</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0:00:15</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>20:18:34</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-001</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Ubada Hussain</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>20:18:49</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-001</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Ubada Hussain</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0:00:15</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>20:19:08</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-001</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Ubada Hussain</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>20:27:20</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-001</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Ubada Hussain</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>20:27:43</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-001</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Ubada Hussain</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>0:00:23</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>20:28:08</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-002</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Ali Raza</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>20:28:23</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>FA24-BSCS-002</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Ali Raza</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>BSCS-1A</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>0:00:15</t>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
change the frame from 2 to 5
</commit_message>
<xml_diff>
--- a/Teacher_Detailed_Attendance.xlsx
+++ b/Teacher_Detailed_Attendance.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -623,7 +623,73 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>04:45:46</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:46:02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Add web page for the Monitering
</commit_message>
<xml_diff>
--- a/Teacher_Detailed_Attendance.xlsx
+++ b/Teacher_Detailed_Attendance.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -689,7 +689,1346 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>20:38:44</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>20:39:02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0:00:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>20:39:23</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>20:51:38</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>20:51:43</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-003</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ustad Gggg</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>20:52:06</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0:00:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>20:52:06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>21:15:24</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>21:16:39</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>21:16:43</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>21:16:54</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0:00:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>21:17:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0:00:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>21:17:09</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>00:49:46</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>00:50:10</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>0:00:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>00:50:19</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>03:22:33</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>03:22:51</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>03:24:39</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>03:25:03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0:00:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>03:25:04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>03:25:17</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BSCS-1A</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>03:33:36</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>03:34:32</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0:00:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>03:34:33</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>03:37:30</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>03:41:26</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>03:41:47</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>03:42:02</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0:00:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>03:42:22</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>03:42:45</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0:00:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>03:42:59</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0:01:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>03:43:08</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>03:43:29</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0:00:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>03:44:14</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>03:44:48</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-001</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Ubada Hussain</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0:00:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>03:45:03</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>03:45:31</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0:00:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>03:45:33</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>FA24-BSCS-002</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Ali Raza</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BSCS-4A</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>